<commit_message>
Update example test file Sorting
Update reference test file for example Sorting. After the style
infrastructure switch, the styles part is saved differently.
</commit_message>
<xml_diff>
--- a/ClosedXML.Tests/Resource/Examples/Ranges/Sorting.xlsx
+++ b/ClosedXML.Tests/Resource/Examples/Ranges/Sorting.xlsx
@@ -61,241 +61,112 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:numFmts count="1">
-    <x:numFmt numFmtId="0" formatCode=""/>
-  </x:numFmts>
-  <x:fonts count="1">
-    <x:font>
-      <x:vertAlign val="baseline"/>
-      <x:sz val="11"/>
-      <x:color rgb="FF000000"/>
-      <x:name val="Calibri"/>
-      <x:family val="2"/>
-    </x:font>
-  </x:fonts>
-  <x:fills count="10">
-    <x:fill>
-      <x:patternFill patternType="none"/>
-    </x:fill>
-    <x:fill>
-      <x:patternFill patternType="gray125"/>
-    </x:fill>
-    <x:fill>
-      <x:patternFill patternType="solid">
-        <x:fgColor rgb="FFDEB887"/>
-      </x:patternFill>
-    </x:fill>
-    <x:fill>
-      <x:patternFill patternType="solid">
-        <x:fgColor rgb="FFA9A9A9"/>
-      </x:patternFill>
-    </x:fill>
-    <x:fill>
-      <x:patternFill patternType="solid">
-        <x:fgColor rgb="FFCD5C5C"/>
-      </x:patternFill>
-    </x:fill>
-    <x:fill>
-      <x:patternFill patternType="solid">
-        <x:fgColor rgb="FF1E90FF"/>
-      </x:patternFill>
-    </x:fill>
-    <x:fill>
-      <x:patternFill patternType="solid">
-        <x:fgColor rgb="FF00CED1"/>
-      </x:patternFill>
-    </x:fill>
-    <x:fill>
-      <x:patternFill patternType="solid">
-        <x:fgColor rgb="FFFF1493"/>
-      </x:patternFill>
-    </x:fill>
-    <x:fill>
-      <x:patternFill patternType="solid">
-        <x:fgColor rgb="FFE9967A"/>
-      </x:patternFill>
-    </x:fill>
-    <x:fill>
-      <x:patternFill patternType="solid">
-        <x:fgColor rgb="FF90EE90"/>
-      </x:patternFill>
-    </x:fill>
-  </x:fills>
-  <x:borders count="1">
-    <x:border diagonalUp="0" diagonalDown="0">
-      <x:left style="none">
-        <x:color rgb="FF000000"/>
-      </x:left>
-      <x:right style="none">
-        <x:color rgb="FF000000"/>
-      </x:right>
-      <x:top style="none">
-        <x:color rgb="FF000000"/>
-      </x:top>
-      <x:bottom style="none">
-        <x:color rgb="FF000000"/>
-      </x:bottom>
-      <x:diagonal style="none">
-        <x:color rgb="FF000000"/>
-      </x:diagonal>
-    </x:border>
-  </x:borders>
-  <x:cellStyleXfs count="21">
-    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyNumberFormat="1" applyFill="1" applyBorder="0" applyAlignment="1" applyProtection="1">
-      <x:protection locked="1" hidden="0"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" applyNumberFormat="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="1">
-      <x:protection locked="1" hidden="0"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="3" borderId="0" applyNumberFormat="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="1">
-      <x:protection locked="1" hidden="0"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="4" borderId="0" applyNumberFormat="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="1">
-      <x:protection locked="1" hidden="0"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="5" borderId="0" applyNumberFormat="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="1">
-      <x:protection locked="1" hidden="0"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="6" borderId="0" applyNumberFormat="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="1">
-      <x:protection locked="1" hidden="0"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="7" borderId="0" applyNumberFormat="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="1">
-      <x:protection locked="1" hidden="0"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="8" borderId="0" applyNumberFormat="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="1">
-      <x:protection locked="1" hidden="0"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="9" borderId="0" applyNumberFormat="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="1">
-      <x:protection locked="1" hidden="0"/>
-    </x:xf>
-    <x:xf numFmtId="46" fontId="0" fillId="4" borderId="0" applyNumberFormat="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="1">
-      <x:protection locked="1" hidden="0"/>
-    </x:xf>
-    <x:xf numFmtId="46" fontId="0" fillId="2" borderId="0" applyNumberFormat="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="1">
-      <x:protection locked="1" hidden="0"/>
-    </x:xf>
-    <x:xf numFmtId="14" fontId="0" fillId="9" borderId="0" applyNumberFormat="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="1">
-      <x:protection locked="1" hidden="0"/>
-    </x:xf>
-    <x:xf numFmtId="14" fontId="0" fillId="7" borderId="0" applyNumberFormat="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="1">
-      <x:protection locked="1" hidden="0"/>
-    </x:xf>
-    <x:xf numFmtId="46" fontId="0" fillId="5" borderId="0" applyNumberFormat="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="1">
-      <x:protection locked="1" hidden="0"/>
-    </x:xf>
-    <x:xf numFmtId="46" fontId="0" fillId="7" borderId="0" applyNumberFormat="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="1">
-      <x:protection locked="1" hidden="0"/>
-    </x:xf>
-    <x:xf numFmtId="46" fontId="0" fillId="9" borderId="0" applyNumberFormat="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="1">
-      <x:protection locked="1" hidden="0"/>
-    </x:xf>
-    <x:xf numFmtId="46" fontId="0" fillId="6" borderId="0" applyNumberFormat="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="1">
-      <x:protection locked="1" hidden="0"/>
-    </x:xf>
-    <x:xf numFmtId="14" fontId="0" fillId="6" borderId="0" applyNumberFormat="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="1">
-      <x:protection locked="1" hidden="0"/>
-    </x:xf>
-    <x:xf numFmtId="14" fontId="0" fillId="4" borderId="0" applyNumberFormat="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="1">
-      <x:protection locked="1" hidden="0"/>
-    </x:xf>
-    <x:xf numFmtId="14" fontId="0" fillId="5" borderId="0" applyNumberFormat="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="1">
-      <x:protection locked="1" hidden="0"/>
-    </x:xf>
-    <x:xf numFmtId="14" fontId="0" fillId="2" borderId="0" applyNumberFormat="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="1">
-      <x:protection locked="1" hidden="0"/>
-    </x:xf>
-  </x:cellStyleXfs>
-  <x:cellXfs count="21">
-    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="0" applyAlignment="1" applyProtection="1">
-      <x:alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <x:protection locked="1" hidden="0"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="1">
-      <x:alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <x:protection locked="1" hidden="0"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="1">
-      <x:alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <x:protection locked="1" hidden="0"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="1">
-      <x:alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <x:protection locked="1" hidden="0"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="1">
-      <x:alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <x:protection locked="1" hidden="0"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="1">
-      <x:alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <x:protection locked="1" hidden="0"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="1">
-      <x:alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <x:protection locked="1" hidden="0"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="1">
-      <x:alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <x:protection locked="1" hidden="0"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="1">
-      <x:alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <x:protection locked="1" hidden="0"/>
-    </x:xf>
-    <x:xf numFmtId="46" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="1">
-      <x:alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <x:protection locked="1" hidden="0"/>
-    </x:xf>
-    <x:xf numFmtId="46" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="1">
-      <x:alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <x:protection locked="1" hidden="0"/>
-    </x:xf>
-    <x:xf numFmtId="14" fontId="0" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="1">
-      <x:alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <x:protection locked="1" hidden="0"/>
-    </x:xf>
-    <x:xf numFmtId="14" fontId="0" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="1">
-      <x:alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <x:protection locked="1" hidden="0"/>
-    </x:xf>
-    <x:xf numFmtId="46" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="1">
-      <x:alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <x:protection locked="1" hidden="0"/>
-    </x:xf>
-    <x:xf numFmtId="46" fontId="0" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="1">
-      <x:alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <x:protection locked="1" hidden="0"/>
-    </x:xf>
-    <x:xf numFmtId="46" fontId="0" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="1">
-      <x:alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <x:protection locked="1" hidden="0"/>
-    </x:xf>
-    <x:xf numFmtId="46" fontId="0" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="1">
-      <x:alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <x:protection locked="1" hidden="0"/>
-    </x:xf>
-    <x:xf numFmtId="14" fontId="0" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="1">
-      <x:alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <x:protection locked="1" hidden="0"/>
-    </x:xf>
-    <x:xf numFmtId="14" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="1">
-      <x:alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <x:protection locked="1" hidden="0"/>
-    </x:xf>
-    <x:xf numFmtId="14" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="1">
-      <x:alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <x:protection locked="1" hidden="0"/>
-    </x:xf>
-    <x:xf numFmtId="14" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="1">
-      <x:alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <x:protection locked="1" hidden="0"/>
-    </x:xf>
-  </x:cellXfs>
-  <x:cellStyles count="1">
-    <x:cellStyle name="Normal" xfId="0" builtinId="0"/>
-  </x:cellStyles>
-</x:styleSheet>
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <fonts count="1">
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+  </fonts>
+  <fills count="10">
+    <fill>
+      <patternFill patternType="none"/>
+    </fill>
+    <fill>
+      <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF90EE90"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF00CED1"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFDEB887"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFA9A9A9"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFE9967A"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF1E90FF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFCD5C5C"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFF1493"/>
+      </patternFill>
+    </fill>
+  </fills>
+  <borders count="1">
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+  </borders>
+  <cellStyleXfs count="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+  </cellStyleXfs>
+  <cellXfs count="21">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="14" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="46" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="46" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="14" fontId="0" fillId="9" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="46" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="46" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="46" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="46" fontId="0" fillId="9" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="14" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="14" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="14" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="14" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1"/>
+  </cellXfs>
+  <cellStyles count="1">
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+  </cellStyles>
+  <dxfs count="0"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
+</styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -604,82 +475,82 @@
       </x:c>
     </x:row>
     <x:row r="2" spans="1:3">
-      <x:c r="A2" s="1" t="s">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="B2" s="1" t="s">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="C2" s="1" t="s">
+      <x:c r="A2" s="3" t="s">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="B2" s="3" t="s">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="C2" s="3" t="s">
         <x:v>5</x:v>
       </x:c>
     </x:row>
     <x:row r="3" spans="1:3">
-      <x:c r="A3" s="2" t="s">
-        <x:v>5</x:v>
-      </x:c>
-      <x:c r="B3" s="2" t="s">
-        <x:v>5</x:v>
-      </x:c>
-      <x:c r="C3" s="2" t="s">
+      <x:c r="A3" s="4" t="s">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="B3" s="4" t="s">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="C3" s="4" t="s">
         <x:v>3</x:v>
       </x:c>
     </x:row>
     <x:row r="4" spans="1:3">
-      <x:c r="A4" s="3" t="s">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="B4" s="3" t="s">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="C4" s="3" t="s">
+      <x:c r="A4" s="7" t="s">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="B4" s="7" t="s">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="C4" s="7" t="s">
         <x:v>5</x:v>
       </x:c>
     </x:row>
     <x:row r="5" spans="1:3">
-      <x:c r="A5" s="4" t="s">
-        <x:v>5</x:v>
-      </x:c>
-      <x:c r="B5" s="4" t="s">
-        <x:v>5</x:v>
-      </x:c>
-      <x:c r="C5" s="4" t="s">
+      <x:c r="A5" s="6" t="s">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="B5" s="6" t="s">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="C5" s="6" t="s">
         <x:v>6</x:v>
       </x:c>
     </x:row>
     <x:row r="6" spans="1:3">
-      <x:c r="A6" s="5" t="s">
-        <x:v>5</x:v>
-      </x:c>
-      <x:c r="B6" s="5" t="s">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="C6" s="5"/>
+      <x:c r="A6" s="2" t="s">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="B6" s="2" t="s">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="C6" s="2"/>
     </x:row>
     <x:row r="7" spans="1:3">
-      <x:c r="A7" s="6" t="s">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="B7" s="6" t="s">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="C7" s="6"/>
+      <x:c r="A7" s="8" t="s">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="B7" s="8" t="s">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="C7" s="8"/>
     </x:row>
     <x:row r="8" spans="1:3">
-      <x:c r="A8" s="7"/>
-      <x:c r="B8" s="7" t="s">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="C8" s="7" t="s">
+      <x:c r="A8" s="5"/>
+      <x:c r="B8" s="5" t="s">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="C8" s="5" t="s">
         <x:v>5</x:v>
       </x:c>
     </x:row>
     <x:row r="9" spans="1:3">
-      <x:c r="A9" s="8" t="s">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="B9" s="8"/>
-      <x:c r="C9" s="8" t="s">
+      <x:c r="A9" s="1" t="s">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="B9" s="1"/>
+      <x:c r="C9" s="1" t="s">
         <x:v>5</x:v>
       </x:c>
     </x:row>
@@ -701,38 +572,38 @@
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:sheetData>
     <x:row r="1" spans="1:1">
-      <x:c r="A1" s="2"/>
+      <x:c r="A1" s="4"/>
     </x:row>
     <x:row r="2" spans="1:1">
-      <x:c r="A2" s="7"/>
+      <x:c r="A2" s="5"/>
     </x:row>
     <x:row r="3" spans="1:1">
-      <x:c r="A3" s="1" t="s">
+      <x:c r="A3" s="3" t="s">
         <x:v>3</x:v>
       </x:c>
     </x:row>
     <x:row r="4" spans="1:1">
-      <x:c r="A4" s="5" t="s">
+      <x:c r="A4" s="2" t="s">
         <x:v>5</x:v>
       </x:c>
     </x:row>
     <x:row r="5" spans="1:1">
-      <x:c r="A5" s="4" t="s">
+      <x:c r="A5" s="6" t="s">
         <x:v>6</x:v>
       </x:c>
     </x:row>
     <x:row r="6" spans="1:1">
-      <x:c r="A6" s="8" t="s">
+      <x:c r="A6" s="1" t="s">
         <x:v>4</x:v>
       </x:c>
     </x:row>
     <x:row r="7" spans="1:1">
-      <x:c r="A7" s="3" t="s">
+      <x:c r="A7" s="7" t="s">
         <x:v>4</x:v>
       </x:c>
     </x:row>
     <x:row r="8" spans="1:1">
-      <x:c r="A8" s="6" t="s">
+      <x:c r="A8" s="8" t="s">
         <x:v>7</x:v>
       </x:c>
     </x:row>
@@ -754,40 +625,40 @@
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:sheetData>
     <x:row r="1" spans="1:1">
-      <x:c r="A1" s="6" t="s">
+      <x:c r="A1" s="8" t="s">
         <x:v>7</x:v>
       </x:c>
     </x:row>
     <x:row r="2" spans="1:1">
-      <x:c r="A2" s="8" t="s">
+      <x:c r="A2" s="1" t="s">
         <x:v>4</x:v>
       </x:c>
     </x:row>
     <x:row r="3" spans="1:1">
-      <x:c r="A3" s="3" t="s">
+      <x:c r="A3" s="7" t="s">
         <x:v>4</x:v>
       </x:c>
     </x:row>
     <x:row r="4" spans="1:1">
-      <x:c r="A4" s="4" t="s">
+      <x:c r="A4" s="6" t="s">
         <x:v>6</x:v>
       </x:c>
     </x:row>
     <x:row r="5" spans="1:1">
-      <x:c r="A5" s="5" t="s">
+      <x:c r="A5" s="2" t="s">
         <x:v>5</x:v>
       </x:c>
     </x:row>
     <x:row r="6" spans="1:1">
-      <x:c r="A6" s="1" t="s">
+      <x:c r="A6" s="3" t="s">
         <x:v>3</x:v>
       </x:c>
     </x:row>
     <x:row r="7" spans="1:1">
-      <x:c r="A7" s="2"/>
+      <x:c r="A7" s="4"/>
     </x:row>
     <x:row r="8" spans="1:1">
-      <x:c r="A8" s="7"/>
+      <x:c r="A8" s="5"/>
     </x:row>
   </x:sheetData>
   <x:printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0"/>
@@ -807,82 +678,82 @@
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:sheetData>
     <x:row r="1" spans="1:3">
-      <x:c r="A1" s="1" t="s">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="B1" s="1" t="s">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="C1" s="1" t="s">
+      <x:c r="A1" s="3" t="s">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="B1" s="3" t="s">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="C1" s="3" t="s">
         <x:v>5</x:v>
       </x:c>
     </x:row>
     <x:row r="2" spans="1:3">
-      <x:c r="A2" s="3" t="s">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="B2" s="3" t="s">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="C2" s="3" t="s">
+      <x:c r="A2" s="7" t="s">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="B2" s="7" t="s">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="C2" s="7" t="s">
         <x:v>5</x:v>
       </x:c>
     </x:row>
     <x:row r="3" spans="1:3">
-      <x:c r="A3" s="2" t="s">
-        <x:v>5</x:v>
-      </x:c>
-      <x:c r="B3" s="2" t="s">
-        <x:v>5</x:v>
-      </x:c>
-      <x:c r="C3" s="2" t="s">
+      <x:c r="A3" s="4" t="s">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="B3" s="4" t="s">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="C3" s="4" t="s">
         <x:v>3</x:v>
       </x:c>
     </x:row>
     <x:row r="4" spans="1:3">
-      <x:c r="A4" s="4" t="s">
-        <x:v>5</x:v>
-      </x:c>
-      <x:c r="B4" s="4" t="s">
-        <x:v>5</x:v>
-      </x:c>
-      <x:c r="C4" s="4" t="s">
+      <x:c r="A4" s="6" t="s">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="B4" s="6" t="s">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="C4" s="6" t="s">
         <x:v>6</x:v>
       </x:c>
     </x:row>
     <x:row r="5" spans="1:3">
-      <x:c r="A5" s="5" t="s">
-        <x:v>5</x:v>
-      </x:c>
-      <x:c r="B5" s="5" t="s">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="C5" s="5"/>
+      <x:c r="A5" s="2" t="s">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="B5" s="2" t="s">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="C5" s="2"/>
     </x:row>
     <x:row r="6" spans="1:3">
-      <x:c r="A6" s="6" t="s">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="B6" s="6" t="s">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="C6" s="6"/>
+      <x:c r="A6" s="8" t="s">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="B6" s="8" t="s">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="C6" s="8"/>
     </x:row>
     <x:row r="7" spans="1:3">
-      <x:c r="A7" s="8" t="s">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="B7" s="8"/>
-      <x:c r="C7" s="8" t="s">
+      <x:c r="A7" s="1" t="s">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="B7" s="1"/>
+      <x:c r="C7" s="1" t="s">
         <x:v>5</x:v>
       </x:c>
     </x:row>
     <x:row r="8" spans="1:3">
-      <x:c r="A8" s="7"/>
-      <x:c r="B8" s="7" t="s">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="C8" s="7" t="s">
+      <x:c r="A8" s="5"/>
+      <x:c r="B8" s="5" t="s">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="C8" s="5" t="s">
         <x:v>5</x:v>
       </x:c>
     </x:row>
@@ -904,40 +775,40 @@
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:sheetData>
     <x:row r="1" spans="1:1">
-      <x:c r="A1" s="1" t="s">
+      <x:c r="A1" s="3" t="s">
         <x:v>3</x:v>
       </x:c>
     </x:row>
     <x:row r="2" spans="1:1">
-      <x:c r="A2" s="5" t="s">
+      <x:c r="A2" s="2" t="s">
         <x:v>5</x:v>
       </x:c>
     </x:row>
     <x:row r="3" spans="1:1">
-      <x:c r="A3" s="4" t="s">
+      <x:c r="A3" s="6" t="s">
         <x:v>6</x:v>
       </x:c>
     </x:row>
     <x:row r="4" spans="1:1">
-      <x:c r="A4" s="8" t="s">
+      <x:c r="A4" s="1" t="s">
         <x:v>4</x:v>
       </x:c>
     </x:row>
     <x:row r="5" spans="1:1">
-      <x:c r="A5" s="3" t="s">
+      <x:c r="A5" s="7" t="s">
         <x:v>4</x:v>
       </x:c>
     </x:row>
     <x:row r="6" spans="1:1">
-      <x:c r="A6" s="6" t="s">
+      <x:c r="A6" s="8" t="s">
         <x:v>7</x:v>
       </x:c>
     </x:row>
     <x:row r="7" spans="1:1">
-      <x:c r="A7" s="2"/>
+      <x:c r="A7" s="4"/>
     </x:row>
     <x:row r="8" spans="1:1">
-      <x:c r="A8" s="7"/>
+      <x:c r="A8" s="5"/>
     </x:row>
   </x:sheetData>
   <x:printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0"/>
@@ -957,40 +828,40 @@
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:sheetData>
     <x:row r="1" spans="1:1">
-      <x:c r="A1" s="6" t="s">
+      <x:c r="A1" s="8" t="s">
         <x:v>7</x:v>
       </x:c>
     </x:row>
     <x:row r="2" spans="1:1">
-      <x:c r="A2" s="8" t="s">
+      <x:c r="A2" s="1" t="s">
         <x:v>4</x:v>
       </x:c>
     </x:row>
     <x:row r="3" spans="1:1">
-      <x:c r="A3" s="3" t="s">
+      <x:c r="A3" s="7" t="s">
         <x:v>4</x:v>
       </x:c>
     </x:row>
     <x:row r="4" spans="1:1">
-      <x:c r="A4" s="4" t="s">
+      <x:c r="A4" s="6" t="s">
         <x:v>6</x:v>
       </x:c>
     </x:row>
     <x:row r="5" spans="1:1">
-      <x:c r="A5" s="5" t="s">
+      <x:c r="A5" s="2" t="s">
         <x:v>5</x:v>
       </x:c>
     </x:row>
     <x:row r="6" spans="1:1">
-      <x:c r="A6" s="1" t="s">
+      <x:c r="A6" s="3" t="s">
         <x:v>3</x:v>
       </x:c>
     </x:row>
     <x:row r="7" spans="1:1">
-      <x:c r="A7" s="2"/>
+      <x:c r="A7" s="4"/>
     </x:row>
     <x:row r="8" spans="1:1">
-      <x:c r="A8" s="7"/>
+      <x:c r="A8" s="5"/>
     </x:row>
   </x:sheetData>
   <x:printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0"/>
@@ -1010,82 +881,82 @@
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:sheetData>
     <x:row r="1" spans="1:3">
-      <x:c r="A1" s="2" t="s">
-        <x:v>5</x:v>
-      </x:c>
-      <x:c r="B1" s="2" t="s">
-        <x:v>5</x:v>
-      </x:c>
-      <x:c r="C1" s="2" t="s">
+      <x:c r="A1" s="4" t="s">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="B1" s="4" t="s">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="C1" s="4" t="s">
         <x:v>3</x:v>
       </x:c>
     </x:row>
     <x:row r="2" spans="1:3">
-      <x:c r="A2" s="3" t="s">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="B2" s="3" t="s">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="C2" s="3" t="s">
+      <x:c r="A2" s="7" t="s">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="B2" s="7" t="s">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="C2" s="7" t="s">
         <x:v>5</x:v>
       </x:c>
     </x:row>
     <x:row r="3" spans="1:3">
-      <x:c r="A3" s="4" t="s">
-        <x:v>5</x:v>
-      </x:c>
-      <x:c r="B3" s="4" t="s">
-        <x:v>5</x:v>
-      </x:c>
-      <x:c r="C3" s="4" t="s">
+      <x:c r="A3" s="6" t="s">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="B3" s="6" t="s">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="C3" s="6" t="s">
         <x:v>6</x:v>
       </x:c>
     </x:row>
     <x:row r="4" spans="1:3">
-      <x:c r="A4" s="5" t="s">
-        <x:v>5</x:v>
-      </x:c>
-      <x:c r="B4" s="5" t="s">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="C4" s="5"/>
+      <x:c r="A4" s="2" t="s">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="B4" s="2" t="s">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="C4" s="2"/>
     </x:row>
     <x:row r="5" spans="1:3">
-      <x:c r="A5" s="1" t="s">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="B5" s="1" t="s">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="C5" s="1" t="s">
+      <x:c r="A5" s="3" t="s">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="B5" s="3" t="s">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="C5" s="3" t="s">
         <x:v>5</x:v>
       </x:c>
     </x:row>
     <x:row r="6" spans="1:3">
-      <x:c r="A6" s="6" t="s">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="B6" s="6" t="s">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="C6" s="6"/>
+      <x:c r="A6" s="8" t="s">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="B6" s="8" t="s">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="C6" s="8"/>
     </x:row>
     <x:row r="7" spans="1:3">
-      <x:c r="A7" s="8" t="s">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="B7" s="8"/>
-      <x:c r="C7" s="8" t="s">
+      <x:c r="A7" s="1" t="s">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="B7" s="1"/>
+      <x:c r="C7" s="1" t="s">
         <x:v>5</x:v>
       </x:c>
     </x:row>
     <x:row r="8" spans="1:3">
-      <x:c r="A8" s="7"/>
-      <x:c r="B8" s="7" t="s">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="C8" s="7" t="s">
+      <x:c r="A8" s="5"/>
+      <x:c r="B8" s="5" t="s">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="C8" s="5" t="s">
         <x:v>5</x:v>
       </x:c>
     </x:row>
@@ -1107,82 +978,82 @@
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:sheetData>
     <x:row r="1" spans="1:3">
-      <x:c r="A1" s="6" t="s">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="B1" s="6" t="s">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="C1" s="6"/>
+      <x:c r="A1" s="8" t="s">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="B1" s="8" t="s">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="C1" s="8"/>
     </x:row>
     <x:row r="2" spans="1:3">
-      <x:c r="A2" s="8" t="s">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="B2" s="8"/>
-      <x:c r="C2" s="8" t="s">
+      <x:c r="A2" s="1" t="s">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="B2" s="1"/>
+      <x:c r="C2" s="1" t="s">
         <x:v>5</x:v>
       </x:c>
     </x:row>
     <x:row r="3" spans="1:3">
-      <x:c r="A3" s="1" t="s">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="B3" s="1" t="s">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="C3" s="1" t="s">
+      <x:c r="A3" s="3" t="s">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="B3" s="3" t="s">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="C3" s="3" t="s">
         <x:v>5</x:v>
       </x:c>
     </x:row>
     <x:row r="4" spans="1:3">
-      <x:c r="A4" s="4" t="s">
-        <x:v>5</x:v>
-      </x:c>
-      <x:c r="B4" s="4" t="s">
-        <x:v>5</x:v>
-      </x:c>
-      <x:c r="C4" s="4" t="s">
+      <x:c r="A4" s="6" t="s">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="B4" s="6" t="s">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="C4" s="6" t="s">
         <x:v>6</x:v>
       </x:c>
     </x:row>
     <x:row r="5" spans="1:3">
-      <x:c r="A5" s="2" t="s">
-        <x:v>5</x:v>
-      </x:c>
-      <x:c r="B5" s="2" t="s">
-        <x:v>5</x:v>
-      </x:c>
-      <x:c r="C5" s="2" t="s">
+      <x:c r="A5" s="4" t="s">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="B5" s="4" t="s">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="C5" s="4" t="s">
         <x:v>3</x:v>
       </x:c>
     </x:row>
     <x:row r="6" spans="1:3">
-      <x:c r="A6" s="3" t="s">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="B6" s="3" t="s">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="C6" s="3" t="s">
+      <x:c r="A6" s="7" t="s">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="B6" s="7" t="s">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="C6" s="7" t="s">
         <x:v>5</x:v>
       </x:c>
     </x:row>
     <x:row r="7" spans="1:3">
-      <x:c r="A7" s="5" t="s">
-        <x:v>5</x:v>
-      </x:c>
-      <x:c r="B7" s="5" t="s">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="C7" s="5"/>
+      <x:c r="A7" s="2" t="s">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="B7" s="2" t="s">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="C7" s="2"/>
     </x:row>
     <x:row r="8" spans="1:3">
-      <x:c r="A8" s="7"/>
-      <x:c r="B8" s="7" t="s">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="C8" s="7" t="s">
+      <x:c r="A8" s="5"/>
+      <x:c r="B8" s="5" t="s">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="C8" s="5" t="s">
         <x:v>5</x:v>
       </x:c>
     </x:row>
@@ -1204,82 +1075,82 @@
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:sheetData>
     <x:row r="1" spans="1:3">
-      <x:c r="A1" s="6" t="s">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="B1" s="6" t="s">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="C1" s="6"/>
+      <x:c r="A1" s="8" t="s">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="B1" s="8" t="s">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="C1" s="8"/>
     </x:row>
     <x:row r="2" spans="1:3">
-      <x:c r="A2" s="2" t="s">
-        <x:v>5</x:v>
-      </x:c>
-      <x:c r="B2" s="2" t="s">
-        <x:v>5</x:v>
-      </x:c>
-      <x:c r="C2" s="2" t="s">
+      <x:c r="A2" s="4" t="s">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="B2" s="4" t="s">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="C2" s="4" t="s">
         <x:v>3</x:v>
       </x:c>
     </x:row>
     <x:row r="3" spans="1:3">
-      <x:c r="A3" s="3" t="s">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="B3" s="3" t="s">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="C3" s="3" t="s">
+      <x:c r="A3" s="7" t="s">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="B3" s="7" t="s">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="C3" s="7" t="s">
         <x:v>5</x:v>
       </x:c>
     </x:row>
     <x:row r="4" spans="1:3">
-      <x:c r="A4" s="4" t="s">
-        <x:v>5</x:v>
-      </x:c>
-      <x:c r="B4" s="4" t="s">
-        <x:v>5</x:v>
-      </x:c>
-      <x:c r="C4" s="4" t="s">
+      <x:c r="A4" s="6" t="s">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="B4" s="6" t="s">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="C4" s="6" t="s">
         <x:v>6</x:v>
       </x:c>
     </x:row>
     <x:row r="5" spans="1:3">
-      <x:c r="A5" s="5" t="s">
-        <x:v>5</x:v>
-      </x:c>
-      <x:c r="B5" s="5" t="s">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="C5" s="5"/>
+      <x:c r="A5" s="2" t="s">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="B5" s="2" t="s">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="C5" s="2"/>
     </x:row>
     <x:row r="6" spans="1:3">
-      <x:c r="A6" s="7"/>
-      <x:c r="B6" s="7" t="s">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="C6" s="7" t="s">
+      <x:c r="A6" s="5"/>
+      <x:c r="B6" s="5" t="s">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="C6" s="5" t="s">
         <x:v>5</x:v>
       </x:c>
     </x:row>
     <x:row r="7" spans="1:3">
-      <x:c r="A7" s="1" t="s">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="B7" s="1" t="s">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="C7" s="1" t="s">
+      <x:c r="A7" s="3" t="s">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="B7" s="3" t="s">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="C7" s="3" t="s">
         <x:v>5</x:v>
       </x:c>
     </x:row>
     <x:row r="8" spans="1:3">
-      <x:c r="A8" s="8" t="s">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="B8" s="8"/>
-      <x:c r="C8" s="8" t="s">
+      <x:c r="A8" s="1" t="s">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="B8" s="1"/>
+      <x:c r="C8" s="1" t="s">
         <x:v>5</x:v>
       </x:c>
     </x:row>
@@ -1301,40 +1172,40 @@
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:sheetData>
     <x:row r="1" spans="1:1">
-      <x:c r="A1" s="5" t="s">
+      <x:c r="A1" s="2" t="s">
         <x:v>5</x:v>
       </x:c>
     </x:row>
     <x:row r="2" spans="1:1">
-      <x:c r="A2" s="1" t="s">
+      <x:c r="A2" s="3" t="s">
         <x:v>3</x:v>
       </x:c>
     </x:row>
     <x:row r="3" spans="1:1">
-      <x:c r="A3" s="8" t="s">
+      <x:c r="A3" s="1" t="s">
         <x:v>4</x:v>
       </x:c>
     </x:row>
     <x:row r="4" spans="1:1">
-      <x:c r="A4" s="4" t="s">
+      <x:c r="A4" s="6" t="s">
         <x:v>6</x:v>
       </x:c>
     </x:row>
     <x:row r="5" spans="1:1">
-      <x:c r="A5" s="3" t="s">
+      <x:c r="A5" s="7" t="s">
         <x:v>4</x:v>
       </x:c>
     </x:row>
     <x:row r="6" spans="1:1">
-      <x:c r="A6" s="6" t="s">
+      <x:c r="A6" s="8" t="s">
         <x:v>7</x:v>
       </x:c>
     </x:row>
     <x:row r="7" spans="1:1">
-      <x:c r="A7" s="2"/>
+      <x:c r="A7" s="4"/>
     </x:row>
     <x:row r="8" spans="1:1">
-      <x:c r="A8" s="7"/>
+      <x:c r="A8" s="5"/>
     </x:row>
   </x:sheetData>
   <x:printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0"/>
@@ -1354,40 +1225,40 @@
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:sheetData>
     <x:row r="1" spans="1:1">
-      <x:c r="A1" s="6" t="s">
+      <x:c r="A1" s="8" t="s">
         <x:v>7</x:v>
       </x:c>
     </x:row>
     <x:row r="2" spans="1:1">
-      <x:c r="A2" s="8" t="s">
+      <x:c r="A2" s="1" t="s">
         <x:v>4</x:v>
       </x:c>
     </x:row>
     <x:row r="3" spans="1:1">
-      <x:c r="A3" s="4" t="s">
+      <x:c r="A3" s="6" t="s">
         <x:v>6</x:v>
       </x:c>
     </x:row>
     <x:row r="4" spans="1:1">
-      <x:c r="A4" s="3" t="s">
+      <x:c r="A4" s="7" t="s">
         <x:v>4</x:v>
       </x:c>
     </x:row>
     <x:row r="5" spans="1:1">
-      <x:c r="A5" s="5" t="s">
+      <x:c r="A5" s="2" t="s">
         <x:v>5</x:v>
       </x:c>
     </x:row>
     <x:row r="6" spans="1:1">
-      <x:c r="A6" s="1" t="s">
+      <x:c r="A6" s="3" t="s">
         <x:v>3</x:v>
       </x:c>
     </x:row>
     <x:row r="7" spans="1:1">
-      <x:c r="A7" s="2"/>
+      <x:c r="A7" s="4"/>
     </x:row>
     <x:row r="8" spans="1:1">
-      <x:c r="A8" s="7"/>
+      <x:c r="A8" s="5"/>
     </x:row>
   </x:sheetData>
   <x:printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0"/>
@@ -1421,82 +1292,82 @@
       </x:c>
     </x:row>
     <x:row r="2" spans="1:3">
-      <x:c r="A2" s="1" t="s">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="B2" s="1" t="s">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="C2" s="1" t="s">
+      <x:c r="A2" s="3" t="s">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="B2" s="3" t="s">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="C2" s="3" t="s">
         <x:v>5</x:v>
       </x:c>
     </x:row>
     <x:row r="3" spans="1:3">
-      <x:c r="A3" s="5" t="s">
-        <x:v>5</x:v>
-      </x:c>
-      <x:c r="B3" s="5" t="s">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="C3" s="5"/>
+      <x:c r="A3" s="2" t="s">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="B3" s="2" t="s">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="C3" s="2"/>
     </x:row>
     <x:row r="4" spans="1:3">
-      <x:c r="A4" s="2" t="s">
-        <x:v>5</x:v>
-      </x:c>
-      <x:c r="B4" s="2" t="s">
-        <x:v>5</x:v>
-      </x:c>
-      <x:c r="C4" s="2" t="s">
+      <x:c r="A4" s="4" t="s">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="B4" s="4" t="s">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="C4" s="4" t="s">
         <x:v>3</x:v>
       </x:c>
     </x:row>
     <x:row r="5" spans="1:3">
-      <x:c r="A5" s="7"/>
-      <x:c r="B5" s="7" t="s">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="C5" s="7" t="s">
+      <x:c r="A5" s="5"/>
+      <x:c r="B5" s="5" t="s">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="C5" s="5" t="s">
         <x:v>5</x:v>
       </x:c>
     </x:row>
     <x:row r="6" spans="1:3">
-      <x:c r="A6" s="4" t="s">
-        <x:v>5</x:v>
-      </x:c>
-      <x:c r="B6" s="4" t="s">
-        <x:v>5</x:v>
-      </x:c>
-      <x:c r="C6" s="4" t="s">
+      <x:c r="A6" s="6" t="s">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="B6" s="6" t="s">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="C6" s="6" t="s">
         <x:v>6</x:v>
       </x:c>
     </x:row>
     <x:row r="7" spans="1:3">
-      <x:c r="A7" s="3" t="s">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="B7" s="3" t="s">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="C7" s="3" t="s">
+      <x:c r="A7" s="7" t="s">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="B7" s="7" t="s">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="C7" s="7" t="s">
         <x:v>5</x:v>
       </x:c>
     </x:row>
     <x:row r="8" spans="1:3">
-      <x:c r="A8" s="6" t="s">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="B8" s="6" t="s">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="C8" s="6"/>
+      <x:c r="A8" s="8" t="s">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="B8" s="8" t="s">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="C8" s="8"/>
     </x:row>
     <x:row r="9" spans="1:3">
-      <x:c r="A9" s="8" t="s">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="B9" s="8"/>
-      <x:c r="C9" s="8" t="s">
+      <x:c r="A9" s="1" t="s">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="B9" s="1"/>
+      <x:c r="C9" s="1" t="s">
         <x:v>5</x:v>
       </x:c>
     </x:row>
@@ -1518,22 +1389,22 @@
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:sheetData>
     <x:row r="1" spans="1:3">
-      <x:c r="A1" s="8" t="s">
-        <x:v>5</x:v>
-      </x:c>
-      <x:c r="B1" s="8" t="s">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="C1" s="8"/>
+      <x:c r="A1" s="1" t="s">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="B1" s="1" t="s">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="C1" s="1"/>
     </x:row>
     <x:row r="2" spans="1:3">
-      <x:c r="A2" s="5" t="s">
-        <x:v>5</x:v>
-      </x:c>
-      <x:c r="B2" s="5" t="s">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="C2" s="5"/>
+      <x:c r="A2" s="2" t="s">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="B2" s="2" t="s">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="C2" s="2"/>
     </x:row>
   </x:sheetData>
   <x:printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0"/>
@@ -1556,64 +1427,64 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1" spans="1:2">
-      <x:c r="A1" s="5" t="s">
-        <x:v>5</x:v>
-      </x:c>
-      <x:c r="B1" s="5" t="s">
+      <x:c r="A1" s="2" t="s">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="B1" s="2" t="s">
         <x:v>3</x:v>
       </x:c>
     </x:row>
     <x:row r="2" spans="1:2">
-      <x:c r="A2" s="1" t="s">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="B2" s="2" t="s">
+      <x:c r="A2" s="3" t="s">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="B2" s="4" t="s">
         <x:v>5</x:v>
       </x:c>
     </x:row>
     <x:row r="3" spans="1:2">
-      <x:c r="A3" s="2" t="s">
-        <x:v>5</x:v>
-      </x:c>
-      <x:c r="B3" s="7" t="s">
+      <x:c r="A3" s="4" t="s">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="B3" s="5" t="s">
         <x:v>3</x:v>
       </x:c>
     </x:row>
     <x:row r="4" spans="1:2">
-      <x:c r="A4" s="4" t="s">
-        <x:v>5</x:v>
-      </x:c>
-      <x:c r="B4" s="4" t="s">
+      <x:c r="A4" s="6" t="s">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="B4" s="6" t="s">
         <x:v>5</x:v>
       </x:c>
     </x:row>
     <x:row r="5" spans="1:2">
-      <x:c r="A5" s="3" t="s">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="B5" s="3" t="s">
+      <x:c r="A5" s="7" t="s">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="B5" s="7" t="s">
         <x:v>3</x:v>
       </x:c>
     </x:row>
     <x:row r="6" spans="1:2">
-      <x:c r="A6" s="8" t="s">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="B6" s="6" t="s">
+      <x:c r="A6" s="1" t="s">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="B6" s="8" t="s">
         <x:v>3</x:v>
       </x:c>
     </x:row>
     <x:row r="7" spans="1:2">
-      <x:c r="A7" s="6" t="s">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="B7" s="1" t="s">
+      <x:c r="A7" s="8" t="s">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="B7" s="3" t="s">
         <x:v>4</x:v>
       </x:c>
     </x:row>
     <x:row r="8" spans="1:2">
-      <x:c r="A8" s="7"/>
-      <x:c r="B8" s="8"/>
+      <x:c r="A8" s="5"/>
+      <x:c r="B8" s="1"/>
     </x:row>
   </x:sheetData>
   <x:printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0"/>
@@ -1633,7 +1504,7 @@
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:sheetData>
     <x:row r="1" spans="1:1">
-      <x:c r="A1" s="9">
+      <x:c r="A1" s="11">
         <x:v>0.378125</x:v>
       </x:c>
     </x:row>
@@ -1643,17 +1514,17 @@
       </x:c>
     </x:row>
     <x:row r="3" spans="1:1">
-      <x:c r="A3" s="5">
+      <x:c r="A3" s="2">
         <x:v>1.15</x:v>
       </x:c>
     </x:row>
     <x:row r="4" spans="1:1">
-      <x:c r="A4" s="4">
+      <x:c r="A4" s="6">
         <x:v>9</x:v>
       </x:c>
     </x:row>
     <x:row r="5" spans="1:1">
-      <x:c r="A5" s="11">
+      <x:c r="A5" s="9">
         <x:v>40573</x:v>
       </x:c>
     </x:row>
@@ -1663,10 +1534,10 @@
       </x:c>
     </x:row>
     <x:row r="7" spans="1:1">
-      <x:c r="A7" s="2"/>
+      <x:c r="A7" s="4"/>
     </x:row>
     <x:row r="8" spans="1:1">
-      <x:c r="A8" s="7"/>
+      <x:c r="A8" s="5"/>
     </x:row>
   </x:sheetData>
   <x:printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0"/>
@@ -1686,40 +1557,40 @@
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:sheetData>
     <x:row r="1" spans="1:1">
-      <x:c r="A1" s="5">
+      <x:c r="A1" s="2">
         <x:v>1.15</x:v>
       </x:c>
     </x:row>
     <x:row r="2" spans="1:1">
-      <x:c r="A2" s="8">
+      <x:c r="A2" s="1">
         <x:v>1.3</x:v>
       </x:c>
     </x:row>
     <x:row r="3" spans="1:1">
-      <x:c r="A3" s="6">
+      <x:c r="A3" s="8">
         <x:v>4.15</x:v>
       </x:c>
     </x:row>
     <x:row r="4" spans="1:1">
-      <x:c r="A4" s="3">
+      <x:c r="A4" s="7">
         <x:v>4.3</x:v>
       </x:c>
     </x:row>
     <x:row r="5" spans="1:1">
-      <x:c r="A5" s="4">
+      <x:c r="A5" s="6">
         <x:v>9</x:v>
       </x:c>
     </x:row>
     <x:row r="6" spans="1:1">
-      <x:c r="A6" s="1">
+      <x:c r="A6" s="3">
         <x:v>1230</x:v>
       </x:c>
     </x:row>
     <x:row r="7" spans="1:1">
-      <x:c r="A7" s="2"/>
+      <x:c r="A7" s="4"/>
     </x:row>
     <x:row r="8" spans="1:1">
-      <x:c r="A8" s="7"/>
+      <x:c r="A8" s="5"/>
     </x:row>
   </x:sheetData>
   <x:printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0"/>
@@ -1739,22 +1610,22 @@
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:sheetData>
     <x:row r="1" spans="1:1">
-      <x:c r="A1" s="13">
+      <x:c r="A1" s="15">
         <x:v>0.00850694444444444</x:v>
       </x:c>
     </x:row>
     <x:row r="2" spans="1:1">
-      <x:c r="A2" s="14">
+      <x:c r="A2" s="16">
         <x:v>0.0446180555555556</x:v>
       </x:c>
     </x:row>
     <x:row r="3" spans="1:1">
-      <x:c r="A3" s="9">
+      <x:c r="A3" s="11">
         <x:v>0.0447916666666667</x:v>
       </x:c>
     </x:row>
     <x:row r="4" spans="1:1">
-      <x:c r="A4" s="15">
+      <x:c r="A4" s="13">
         <x:v>0.524548611111111</x:v>
       </x:c>
     </x:row>
@@ -1764,15 +1635,15 @@
       </x:c>
     </x:row>
     <x:row r="6" spans="1:1">
-      <x:c r="A6" s="16">
+      <x:c r="A6" s="14">
         <x:v>1.87586805555556</x:v>
       </x:c>
     </x:row>
     <x:row r="7" spans="1:1">
-      <x:c r="A7" s="2"/>
+      <x:c r="A7" s="4"/>
     </x:row>
     <x:row r="8" spans="1:1">
-      <x:c r="A8" s="7"/>
+      <x:c r="A8" s="5"/>
     </x:row>
   </x:sheetData>
   <x:printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0"/>
@@ -1797,7 +1668,7 @@
       </x:c>
     </x:row>
     <x:row r="2" spans="1:1">
-      <x:c r="A2" s="11">
+      <x:c r="A2" s="9">
         <x:v>40573</x:v>
       </x:c>
     </x:row>
@@ -1807,7 +1678,7 @@
       </x:c>
     </x:row>
     <x:row r="4" spans="1:1">
-      <x:c r="A4" s="18">
+      <x:c r="A4" s="20">
         <x:v>40663</x:v>
       </x:c>
     </x:row>
@@ -1817,15 +1688,15 @@
       </x:c>
     </x:row>
     <x:row r="6" spans="1:1">
-      <x:c r="A6" s="20">
+      <x:c r="A6" s="18">
         <x:v>40907</x:v>
       </x:c>
     </x:row>
     <x:row r="7" spans="1:1">
-      <x:c r="A7" s="2"/>
+      <x:c r="A7" s="4"/>
     </x:row>
     <x:row r="8" spans="1:1">
-      <x:c r="A8" s="7"/>
+      <x:c r="A8" s="5"/>
     </x:row>
   </x:sheetData>
   <x:printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0"/>
@@ -1845,82 +1716,82 @@
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:sheetData>
     <x:row r="1" spans="1:3">
-      <x:c r="A1" s="7"/>
-      <x:c r="B1" s="7" t="s">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="C1" s="7" t="s">
+      <x:c r="A1" s="5"/>
+      <x:c r="B1" s="5" t="s">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="C1" s="5" t="s">
         <x:v>5</x:v>
       </x:c>
     </x:row>
     <x:row r="2" spans="1:3">
-      <x:c r="A2" s="1" t="s">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="B2" s="1" t="s">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="C2" s="1" t="s">
+      <x:c r="A2" s="3" t="s">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="B2" s="3" t="s">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="C2" s="3" t="s">
         <x:v>5</x:v>
       </x:c>
     </x:row>
     <x:row r="3" spans="1:3">
-      <x:c r="A3" s="3" t="s">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="B3" s="3" t="s">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="C3" s="3" t="s">
+      <x:c r="A3" s="7" t="s">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="B3" s="7" t="s">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="C3" s="7" t="s">
         <x:v>5</x:v>
       </x:c>
     </x:row>
     <x:row r="4" spans="1:3">
-      <x:c r="A4" s="2" t="s">
-        <x:v>5</x:v>
-      </x:c>
-      <x:c r="B4" s="2" t="s">
-        <x:v>5</x:v>
-      </x:c>
-      <x:c r="C4" s="2" t="s">
+      <x:c r="A4" s="4" t="s">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="B4" s="4" t="s">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="C4" s="4" t="s">
         <x:v>3</x:v>
       </x:c>
     </x:row>
     <x:row r="5" spans="1:3">
-      <x:c r="A5" s="4" t="s">
-        <x:v>5</x:v>
-      </x:c>
-      <x:c r="B5" s="4" t="s">
-        <x:v>5</x:v>
-      </x:c>
-      <x:c r="C5" s="4" t="s">
+      <x:c r="A5" s="6" t="s">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="B5" s="6" t="s">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="C5" s="6" t="s">
         <x:v>6</x:v>
       </x:c>
     </x:row>
     <x:row r="6" spans="1:3">
-      <x:c r="A6" s="5" t="s">
-        <x:v>5</x:v>
-      </x:c>
-      <x:c r="B6" s="5" t="s">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="C6" s="5"/>
+      <x:c r="A6" s="2" t="s">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="B6" s="2" t="s">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="C6" s="2"/>
     </x:row>
     <x:row r="7" spans="1:3">
-      <x:c r="A7" s="6" t="s">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="B7" s="6" t="s">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="C7" s="6"/>
+      <x:c r="A7" s="8" t="s">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="B7" s="8" t="s">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="C7" s="8"/>
     </x:row>
     <x:row r="8" spans="1:3">
-      <x:c r="A8" s="8" t="s">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="B8" s="8"/>
-      <x:c r="C8" s="8" t="s">
+      <x:c r="A8" s="1" t="s">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="B8" s="1"/>
+      <x:c r="C8" s="1" t="s">
         <x:v>5</x:v>
       </x:c>
     </x:row>

</xml_diff>